<commit_message>
Part way through changing setup script to include factors
</commit_message>
<xml_diff>
--- a/WVS_Dataset/WVS7_Variable_Index.xlsx
+++ b/WVS_Dataset/WVS7_Variable_Index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\file\Usersj$\jwa349\Home\My Documents\GitHub\PSYC382_WVS7_Shiny\WVS_Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBAC076D-ADAA-4671-B550-9EE5FBFC6EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D1D4FA-91A5-4843-BBEF-48F099E655B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21580" yWindow="12570" windowWidth="21760" windowHeight="18860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="260" yWindow="13000" windowWidth="21760" windowHeight="18860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4969" uniqueCount="2165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4969" uniqueCount="2166">
   <si>
     <t>Col_ID</t>
   </si>
@@ -6518,6 +6518,9 @@
   </si>
   <si>
     <t>Q289-Religious affiliation</t>
+  </si>
+  <si>
+    <t>ordinal</t>
   </si>
 </sst>
 </file>
@@ -6870,6 +6873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:T318"/>
   <sheetFormatPr defaultColWidth="28.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -6935,7 +6939,7 @@
         <v>2088</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -6982,7 +6986,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -7032,7 +7036,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -7088,7 +7092,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>49</v>
       </c>
@@ -7144,7 +7148,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -7200,7 +7204,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>63</v>
       </c>
@@ -7256,7 +7260,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>70</v>
       </c>
@@ -7312,7 +7316,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -7368,7 +7372,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>84</v>
       </c>
@@ -7424,7 +7428,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>93</v>
       </c>
@@ -7480,7 +7484,7 @@
         <v>2089</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>101</v>
       </c>
@@ -7536,7 +7540,7 @@
         <v>2090</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2070</v>
       </c>
@@ -7565,7 +7569,7 @@
         <v>2091</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>111</v>
       </c>
@@ -7621,7 +7625,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>2071</v>
       </c>
@@ -7650,7 +7654,7 @@
         <v>2092</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>118</v>
       </c>
@@ -7706,7 +7710,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>2072</v>
       </c>
@@ -7735,7 +7739,7 @@
         <v>2093</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>125</v>
       </c>
@@ -7791,7 +7795,7 @@
         <v>2094</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>2073</v>
       </c>
@@ -7820,7 +7824,7 @@
         <v>2095</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>132</v>
       </c>
@@ -7876,7 +7880,7 @@
         <v>2096</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>2074</v>
       </c>
@@ -7905,7 +7909,7 @@
         <v>2097</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>140</v>
       </c>
@@ -7961,7 +7965,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>2075</v>
       </c>
@@ -7990,7 +7994,7 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>147</v>
       </c>
@@ -8052,7 +8056,7 @@
         <v>2099</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>160</v>
       </c>
@@ -8114,7 +8118,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>168</v>
       </c>
@@ -8176,7 +8180,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>176</v>
       </c>
@@ -8238,7 +8242,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>184</v>
       </c>
@@ -8294,7 +8298,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>189</v>
       </c>
@@ -8356,7 +8360,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>199</v>
       </c>
@@ -8418,7 +8422,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>208</v>
       </c>
@@ -8480,7 +8484,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>218</v>
       </c>
@@ -8536,7 +8540,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>227</v>
       </c>
@@ -8592,7 +8596,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>233</v>
       </c>
@@ -8648,7 +8652,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>239</v>
       </c>
@@ -8704,7 +8708,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>245</v>
       </c>
@@ -8760,7 +8764,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>251</v>
       </c>
@@ -8813,7 +8817,7 @@
         <v>2101</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>259</v>
       </c>
@@ -8866,7 +8870,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>267</v>
       </c>
@@ -8922,7 +8926,7 @@
         <v>2102</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>273</v>
       </c>
@@ -8981,7 +8985,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>283</v>
       </c>
@@ -9034,7 +9038,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>292</v>
       </c>
@@ -9090,7 +9094,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>301</v>
       </c>
@@ -9146,7 +9150,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>307</v>
       </c>
@@ -9202,7 +9206,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>313</v>
       </c>
@@ -9258,7 +9262,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>319</v>
       </c>
@@ -9314,7 +9318,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>325</v>
       </c>
@@ -9370,7 +9374,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>331</v>
       </c>
@@ -9426,7 +9430,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>337</v>
       </c>
@@ -9482,7 +9486,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>343</v>
       </c>
@@ -9538,7 +9542,7 @@
         <v>2103</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>348</v>
       </c>
@@ -9591,7 +9595,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>355</v>
       </c>
@@ -9644,7 +9648,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>364</v>
       </c>
@@ -9700,7 +9704,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>373</v>
       </c>
@@ -9756,7 +9760,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>379</v>
       </c>
@@ -9812,7 +9816,7 @@
         <v>2104</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>385</v>
       </c>
@@ -9868,7 +9872,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>391</v>
       </c>
@@ -9924,7 +9928,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>397</v>
       </c>
@@ -9980,7 +9984,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>403</v>
       </c>
@@ -10036,7 +10040,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>409</v>
       </c>
@@ -10092,7 +10096,7 @@
         <v>2105</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>419</v>
       </c>
@@ -10148,7 +10152,7 @@
         <v>2106</v>
       </c>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>424</v>
       </c>
@@ -10204,7 +10208,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>430</v>
       </c>
@@ -10260,7 +10264,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>436</v>
       </c>
@@ -10316,7 +10320,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>445</v>
       </c>
@@ -10372,7 +10376,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>451</v>
       </c>
@@ -10428,7 +10432,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>458</v>
       </c>
@@ -10484,7 +10488,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>463</v>
       </c>
@@ -10540,7 +10544,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>469</v>
       </c>
@@ -10596,7 +10600,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>475</v>
       </c>
@@ -10652,7 +10656,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>482</v>
       </c>
@@ -10705,7 +10709,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>489</v>
       </c>
@@ -10761,7 +10765,7 @@
         <v>2107</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>494</v>
       </c>
@@ -10814,7 +10818,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>500</v>
       </c>
@@ -10867,7 +10871,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>506</v>
       </c>
@@ -10923,7 +10927,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>516</v>
       </c>
@@ -10979,7 +10983,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>523</v>
       </c>
@@ -11032,7 +11036,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>530</v>
       </c>
@@ -11085,7 +11089,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>537</v>
       </c>
@@ -11138,7 +11142,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>544</v>
       </c>
@@ -11191,7 +11195,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>551</v>
       </c>
@@ -11253,7 +11257,7 @@
         <v>2108</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>563</v>
       </c>
@@ -11315,7 +11319,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>570</v>
       </c>
@@ -11371,7 +11375,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>576</v>
       </c>
@@ -11433,7 +11437,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>582</v>
       </c>
@@ -11495,7 +11499,7 @@
         <v>2110</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>588</v>
       </c>
@@ -11557,7 +11561,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>594</v>
       </c>
@@ -11616,7 +11620,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>604</v>
       </c>
@@ -11692,7 +11696,7 @@
         <v>618</v>
       </c>
       <c r="G89" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="H89" t="s">
         <v>619</v>
@@ -11707,7 +11711,7 @@
         <v>22</v>
       </c>
       <c r="L89" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="M89" t="s">
         <v>618</v>
@@ -11748,7 +11752,7 @@
         <v>625</v>
       </c>
       <c r="G90" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="H90" t="s">
         <v>619</v>
@@ -11763,7 +11767,7 @@
         <v>22</v>
       </c>
       <c r="L90" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="M90" t="s">
         <v>625</v>
@@ -11804,7 +11808,7 @@
         <v>631</v>
       </c>
       <c r="G91" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="H91" t="s">
         <v>619</v>
@@ -11819,7 +11823,7 @@
         <v>22</v>
       </c>
       <c r="L91" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="M91" t="s">
         <v>631</v>
@@ -11860,7 +11864,7 @@
         <v>637</v>
       </c>
       <c r="G92" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="H92" t="s">
         <v>619</v>
@@ -11875,7 +11879,7 @@
         <v>22</v>
       </c>
       <c r="L92" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="M92" t="s">
         <v>637</v>
@@ -11899,7 +11903,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>641</v>
       </c>
@@ -11955,7 +11959,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>649</v>
       </c>
@@ -12011,7 +12015,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>654</v>
       </c>
@@ -12067,7 +12071,7 @@
         <v>2113</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>659</v>
       </c>
@@ -12120,7 +12124,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>667</v>
       </c>
@@ -12173,7 +12177,7 @@
         <v>2114</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>2076</v>
       </c>
@@ -12199,7 +12203,7 @@
         <v>2115</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>674</v>
       </c>
@@ -12252,7 +12256,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>682</v>
       </c>
@@ -12305,7 +12309,7 @@
         <v>2116</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>690</v>
       </c>
@@ -12358,7 +12362,7 @@
         <v>2117</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>698</v>
       </c>
@@ -12437,7 +12441,7 @@
         <v>712</v>
       </c>
       <c r="G103" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H103" t="s">
         <v>619</v>
@@ -12452,7 +12456,7 @@
         <v>153</v>
       </c>
       <c r="L103" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M103" t="s">
         <v>712</v>
@@ -12499,7 +12503,7 @@
         <v>720</v>
       </c>
       <c r="G104" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H104" t="s">
         <v>619</v>
@@ -12514,7 +12518,7 @@
         <v>153</v>
       </c>
       <c r="L104" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M104" t="s">
         <v>720</v>
@@ -12561,7 +12565,7 @@
         <v>726</v>
       </c>
       <c r="G105" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H105" t="s">
         <v>619</v>
@@ -12576,7 +12580,7 @@
         <v>153</v>
       </c>
       <c r="L105" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M105" t="s">
         <v>726</v>
@@ -12603,7 +12607,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>730</v>
       </c>
@@ -12679,7 +12683,7 @@
         <v>740</v>
       </c>
       <c r="G107" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H107" t="s">
         <v>619</v>
@@ -12694,7 +12698,7 @@
         <v>153</v>
       </c>
       <c r="L107" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M107" t="s">
         <v>740</v>
@@ -12741,7 +12745,7 @@
         <v>746</v>
       </c>
       <c r="G108" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H108" t="s">
         <v>619</v>
@@ -12756,7 +12760,7 @@
         <v>153</v>
       </c>
       <c r="L108" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M108" t="s">
         <v>746</v>
@@ -12803,7 +12807,7 @@
         <v>752</v>
       </c>
       <c r="G109" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H109" t="s">
         <v>619</v>
@@ -12818,7 +12822,7 @@
         <v>153</v>
       </c>
       <c r="L109" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M109" t="s">
         <v>752</v>
@@ -12865,7 +12869,7 @@
         <v>758</v>
       </c>
       <c r="G110" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H110" t="s">
         <v>619</v>
@@ -12880,7 +12884,7 @@
         <v>153</v>
       </c>
       <c r="L110" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M110" t="s">
         <v>758</v>
@@ -12927,7 +12931,7 @@
         <v>764</v>
       </c>
       <c r="G111" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H111" t="s">
         <v>619</v>
@@ -12942,7 +12946,7 @@
         <v>153</v>
       </c>
       <c r="L111" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M111" t="s">
         <v>764</v>
@@ -12989,7 +12993,7 @@
         <v>770</v>
       </c>
       <c r="G112" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H112" t="s">
         <v>619</v>
@@ -13004,7 +13008,7 @@
         <v>153</v>
       </c>
       <c r="L112" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M112" t="s">
         <v>770</v>
@@ -13051,7 +13055,7 @@
         <v>776</v>
       </c>
       <c r="G113" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H113" t="s">
         <v>619</v>
@@ -13066,7 +13070,7 @@
         <v>153</v>
       </c>
       <c r="L113" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M113" t="s">
         <v>776</v>
@@ -13113,7 +13117,7 @@
         <v>782</v>
       </c>
       <c r="G114" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H114" t="s">
         <v>619</v>
@@ -13128,7 +13132,7 @@
         <v>153</v>
       </c>
       <c r="L114" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M114" t="s">
         <v>782</v>
@@ -13175,7 +13179,7 @@
         <v>788</v>
       </c>
       <c r="G115" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H115" t="s">
         <v>619</v>
@@ -13190,7 +13194,7 @@
         <v>153</v>
       </c>
       <c r="L115" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M115" t="s">
         <v>788</v>
@@ -13237,7 +13241,7 @@
         <v>794</v>
       </c>
       <c r="G116" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H116" t="s">
         <v>619</v>
@@ -13252,7 +13256,7 @@
         <v>153</v>
       </c>
       <c r="L116" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M116" t="s">
         <v>794</v>
@@ -13279,7 +13283,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>798</v>
       </c>
@@ -13355,7 +13359,7 @@
         <v>805</v>
       </c>
       <c r="G118" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H118" t="s">
         <v>619</v>
@@ -13370,7 +13374,7 @@
         <v>153</v>
       </c>
       <c r="L118" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M118" t="s">
         <v>805</v>
@@ -13417,7 +13421,7 @@
         <v>811</v>
       </c>
       <c r="G119" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H119" t="s">
         <v>619</v>
@@ -13432,7 +13436,7 @@
         <v>153</v>
       </c>
       <c r="L119" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M119" t="s">
         <v>811</v>
@@ -13479,7 +13483,7 @@
         <v>817</v>
       </c>
       <c r="G120" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H120" t="s">
         <v>619</v>
@@ -13494,7 +13498,7 @@
         <v>153</v>
       </c>
       <c r="L120" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M120" t="s">
         <v>817</v>
@@ -13541,7 +13545,7 @@
         <v>823</v>
       </c>
       <c r="G121" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H121" t="s">
         <v>619</v>
@@ -13556,7 +13560,7 @@
         <v>153</v>
       </c>
       <c r="L121" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M121" t="s">
         <v>823</v>
@@ -13603,7 +13607,7 @@
         <v>829</v>
       </c>
       <c r="G122" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H122" t="s">
         <v>619</v>
@@ -13618,7 +13622,7 @@
         <v>153</v>
       </c>
       <c r="L122" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M122" t="s">
         <v>829</v>
@@ -13665,7 +13669,7 @@
         <v>836</v>
       </c>
       <c r="G123" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H123" t="s">
         <v>619</v>
@@ -13680,7 +13684,7 @@
         <v>153</v>
       </c>
       <c r="L123" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M123" t="s">
         <v>836</v>
@@ -13707,7 +13711,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>840</v>
       </c>
@@ -13763,7 +13767,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>849</v>
       </c>
@@ -13819,7 +13823,7 @@
         <v>2119</v>
       </c>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>855</v>
       </c>
@@ -13875,7 +13879,7 @@
         <v>2120</v>
       </c>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>862</v>
       </c>
@@ -13928,7 +13932,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>870</v>
       </c>
@@ -13984,7 +13988,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>875</v>
       </c>
@@ -14040,7 +14044,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>880</v>
       </c>
@@ -14093,7 +14097,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>887</v>
       </c>
@@ -14149,7 +14153,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>896</v>
       </c>
@@ -14205,7 +14209,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>903</v>
       </c>
@@ -14261,7 +14265,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>909</v>
       </c>
@@ -14317,7 +14321,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>915</v>
       </c>
@@ -14373,7 +14377,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>921</v>
       </c>
@@ -14429,7 +14433,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>927</v>
       </c>
@@ -14485,7 +14489,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>933</v>
       </c>
@@ -14541,7 +14545,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>939</v>
       </c>
@@ -14597,7 +14601,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>948</v>
       </c>
@@ -14653,7 +14657,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>953</v>
       </c>
@@ -14709,7 +14713,7 @@
         <v>2121</v>
       </c>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>960</v>
       </c>
@@ -14765,7 +14769,7 @@
         <v>2122</v>
       </c>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>966</v>
       </c>
@@ -14821,7 +14825,7 @@
         <v>2123</v>
       </c>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>973</v>
       </c>
@@ -14877,7 +14881,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="145" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>980</v>
       </c>
@@ -14933,7 +14937,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="146" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>986</v>
       </c>
@@ -14989,7 +14993,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="147" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>992</v>
       </c>
@@ -15045,7 +15049,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="148" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>998</v>
       </c>
@@ -15101,7 +15105,7 @@
         <v>2124</v>
       </c>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>1006</v>
       </c>
@@ -15157,7 +15161,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="150" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>1012</v>
       </c>
@@ -15213,7 +15217,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="151" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>1018</v>
       </c>
@@ -15269,7 +15273,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="152" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>1023</v>
       </c>
@@ -15325,7 +15329,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="153" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>1029</v>
       </c>
@@ -15381,7 +15385,7 @@
         <v>1033</v>
       </c>
     </row>
-    <row r="154" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>1038</v>
       </c>
@@ -15437,7 +15441,7 @@
         <v>2125</v>
       </c>
     </row>
-    <row r="155" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>1044</v>
       </c>
@@ -15493,7 +15497,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="156" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>1052</v>
       </c>
@@ -15549,7 +15553,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="157" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>1061</v>
       </c>
@@ -15605,7 +15609,7 @@
         <v>2126</v>
       </c>
     </row>
-    <row r="158" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>1068</v>
       </c>
@@ -15661,7 +15665,7 @@
         <v>1071</v>
       </c>
     </row>
-    <row r="159" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>1074</v>
       </c>
@@ -15717,7 +15721,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="160" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>1080</v>
       </c>
@@ -15773,7 +15777,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="161" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>1086</v>
       </c>
@@ -15829,7 +15833,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="162" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>1092</v>
       </c>
@@ -15885,7 +15889,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="163" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>1097</v>
       </c>
@@ -15941,7 +15945,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="164" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>1103</v>
       </c>
@@ -15997,7 +16001,7 @@
         <v>2127</v>
       </c>
     </row>
-    <row r="165" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>1109</v>
       </c>
@@ -16053,7 +16057,7 @@
         <v>2128</v>
       </c>
     </row>
-    <row r="166" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>1115</v>
       </c>
@@ -16109,7 +16113,7 @@
         <v>2129</v>
       </c>
     </row>
-    <row r="167" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>1121</v>
       </c>
@@ -16162,7 +16166,7 @@
         <v>2130</v>
       </c>
     </row>
-    <row r="168" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>1129</v>
       </c>
@@ -16218,7 +16222,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="169" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>1139</v>
       </c>
@@ -16274,7 +16278,7 @@
         <v>2132</v>
       </c>
     </row>
-    <row r="170" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>1145</v>
       </c>
@@ -16330,7 +16334,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="171" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>1151</v>
       </c>
@@ -16386,7 +16390,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="172" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>1157</v>
       </c>
@@ -16442,7 +16446,7 @@
         <v>2133</v>
       </c>
     </row>
-    <row r="173" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>1165</v>
       </c>
@@ -16498,7 +16502,7 @@
         <v>1167</v>
       </c>
     </row>
-    <row r="174" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>1170</v>
       </c>
@@ -16557,7 +16561,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="175" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>1178</v>
       </c>
@@ -16619,7 +16623,7 @@
         <v>1183</v>
       </c>
     </row>
-    <row r="176" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>1189</v>
       </c>
@@ -16681,7 +16685,7 @@
         <v>1192</v>
       </c>
     </row>
-    <row r="177" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>1195</v>
       </c>
@@ -16743,7 +16747,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="178" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>1202</v>
       </c>
@@ -16805,7 +16809,7 @@
         <v>1205</v>
       </c>
     </row>
-    <row r="179" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>1208</v>
       </c>
@@ -16867,7 +16871,7 @@
         <v>1211</v>
       </c>
     </row>
-    <row r="180" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>1214</v>
       </c>
@@ -16929,7 +16933,7 @@
         <v>2134</v>
       </c>
     </row>
-    <row r="181" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>1220</v>
       </c>
@@ -16991,7 +16995,7 @@
         <v>1223</v>
       </c>
     </row>
-    <row r="182" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>1226</v>
       </c>
@@ -17053,7 +17057,7 @@
         <v>1229</v>
       </c>
     </row>
-    <row r="183" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>1232</v>
       </c>
@@ -17115,7 +17119,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>1238</v>
       </c>
@@ -17171,7 +17175,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="185" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>1243</v>
       </c>
@@ -17230,7 +17234,7 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="186" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>1253</v>
       </c>
@@ -17289,7 +17293,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="187" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>1263</v>
       </c>
@@ -17348,7 +17352,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="188" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>1273</v>
       </c>
@@ -17401,7 +17405,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="189" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>1281</v>
       </c>
@@ -17460,7 +17464,7 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="190" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>1290</v>
       </c>
@@ -17522,7 +17526,7 @@
         <v>1294</v>
       </c>
     </row>
-    <row r="191" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>1299</v>
       </c>
@@ -17584,7 +17588,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="192" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>1305</v>
       </c>
@@ -17646,7 +17650,7 @@
         <v>1308</v>
       </c>
     </row>
-    <row r="193" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>1311</v>
       </c>
@@ -17708,7 +17712,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="194" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>1317</v>
       </c>
@@ -17770,7 +17774,7 @@
         <v>1320</v>
       </c>
     </row>
-    <row r="195" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>1324</v>
       </c>
@@ -17840,7 +17844,7 @@
         <v>1332</v>
       </c>
       <c r="G196" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="H196" t="s">
         <v>619</v>
@@ -17855,7 +17859,7 @@
         <v>22</v>
       </c>
       <c r="L196" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="M196" t="s">
         <v>1332</v>
@@ -17879,7 +17883,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="197" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>1337</v>
       </c>
@@ -17946,7 +17950,7 @@
         <v>1346</v>
       </c>
       <c r="G198" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H198" t="s">
         <v>619</v>
@@ -17961,7 +17965,7 @@
         <v>153</v>
       </c>
       <c r="L198" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M198" t="s">
         <v>1346</v>
@@ -17999,7 +18003,7 @@
         <v>1353</v>
       </c>
       <c r="G199" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="H199" t="s">
         <v>619</v>
@@ -18014,7 +18018,7 @@
         <v>22</v>
       </c>
       <c r="L199" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="M199" t="s">
         <v>1353</v>
@@ -18038,7 +18042,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="200" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>1359</v>
       </c>
@@ -18091,7 +18095,7 @@
         <v>1362</v>
       </c>
     </row>
-    <row r="201" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>1367</v>
       </c>
@@ -18144,7 +18148,7 @@
         <v>1370</v>
       </c>
     </row>
-    <row r="202" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>1374</v>
       </c>
@@ -18194,7 +18198,7 @@
         <v>1378</v>
       </c>
     </row>
-    <row r="203" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>1381</v>
       </c>
@@ -18244,7 +18248,7 @@
         <v>1385</v>
       </c>
     </row>
-    <row r="204" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>1388</v>
       </c>
@@ -18294,7 +18298,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="205" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>1395</v>
       </c>
@@ -18347,7 +18351,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="206" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>1401</v>
       </c>
@@ -18403,7 +18407,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="207" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>1409</v>
       </c>
@@ -18456,7 +18460,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="208" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>1417</v>
       </c>
@@ -18509,7 +18513,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="209" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>1425</v>
       </c>
@@ -18565,7 +18569,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="210" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>1431</v>
       </c>
@@ -18618,7 +18622,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="211" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>1439</v>
       </c>
@@ -18700,7 +18704,7 @@
         <v>41</v>
       </c>
       <c r="L212" t="s">
-        <v>42</v>
+        <v>2165</v>
       </c>
       <c r="M212" t="s">
         <v>1449</v>
@@ -18724,7 +18728,7 @@
         <v>1450</v>
       </c>
     </row>
-    <row r="213" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>2077</v>
       </c>
@@ -18750,7 +18754,7 @@
         <v>2135</v>
       </c>
     </row>
-    <row r="214" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>1454</v>
       </c>
@@ -18803,7 +18807,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="215" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>2078</v>
       </c>
@@ -18829,7 +18833,7 @@
         <v>2136</v>
       </c>
     </row>
-    <row r="216" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>1461</v>
       </c>
@@ -18882,7 +18886,7 @@
         <v>1464</v>
       </c>
     </row>
-    <row r="217" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>2079</v>
       </c>
@@ -18908,7 +18912,7 @@
         <v>2137</v>
       </c>
     </row>
-    <row r="218" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>1467</v>
       </c>
@@ -18961,7 +18965,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="219" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>2080</v>
       </c>
@@ -18987,7 +18991,7 @@
         <v>2138</v>
       </c>
     </row>
-    <row r="220" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>1473</v>
       </c>
@@ -19040,7 +19044,7 @@
         <v>1476</v>
       </c>
     </row>
-    <row r="221" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>1481</v>
       </c>
@@ -19096,7 +19100,7 @@
         <v>1483</v>
       </c>
     </row>
-    <row r="222" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>1486</v>
       </c>
@@ -19149,7 +19153,7 @@
         <v>1489</v>
       </c>
     </row>
-    <row r="223" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>1493</v>
       </c>
@@ -19202,7 +19206,7 @@
         <v>1496</v>
       </c>
     </row>
-    <row r="224" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>1500</v>
       </c>
@@ -19255,7 +19259,7 @@
         <v>1503</v>
       </c>
     </row>
-    <row r="225" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>1506</v>
       </c>
@@ -19308,7 +19312,7 @@
         <v>1509</v>
       </c>
     </row>
-    <row r="226" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>1511</v>
       </c>
@@ -19361,7 +19365,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="227" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>1519</v>
       </c>
@@ -19414,7 +19418,7 @@
         <v>1522</v>
       </c>
     </row>
-    <row r="228" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>1524</v>
       </c>
@@ -19467,7 +19471,7 @@
         <v>1527</v>
       </c>
     </row>
-    <row r="229" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>1532</v>
       </c>
@@ -19537,7 +19541,7 @@
         <v>1543</v>
       </c>
       <c r="G230" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="H230" t="s">
         <v>619</v>
@@ -19552,7 +19556,7 @@
         <v>153</v>
       </c>
       <c r="L230" t="s">
-        <v>154</v>
+        <v>2165</v>
       </c>
       <c r="M230" t="s">
         <v>1543</v>
@@ -19579,7 +19583,7 @@
         <v>1544</v>
       </c>
     </row>
-    <row r="231" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>2081</v>
       </c>
@@ -19664,7 +19668,7 @@
         <v>2140</v>
       </c>
     </row>
-    <row r="233" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>1552</v>
       </c>
@@ -19720,7 +19724,7 @@
         <v>1554</v>
       </c>
     </row>
-    <row r="234" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>1557</v>
       </c>
@@ -19773,7 +19777,7 @@
         <v>2141</v>
       </c>
     </row>
-    <row r="235" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>1565</v>
       </c>
@@ -19829,7 +19833,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="236" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>1570</v>
       </c>
@@ -19885,7 +19889,7 @@
         <v>1572</v>
       </c>
     </row>
-    <row r="237" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>1575</v>
       </c>
@@ -19941,7 +19945,7 @@
         <v>1577</v>
       </c>
     </row>
-    <row r="238" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>1581</v>
       </c>
@@ -19997,7 +20001,7 @@
         <v>1583</v>
       </c>
     </row>
-    <row r="239" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>1586</v>
       </c>
@@ -20053,7 +20057,7 @@
         <v>1589</v>
       </c>
     </row>
-    <row r="240" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>1594</v>
       </c>
@@ -20109,7 +20113,7 @@
         <v>1596</v>
       </c>
     </row>
-    <row r="241" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>1600</v>
       </c>
@@ -20165,7 +20169,7 @@
         <v>1602</v>
       </c>
     </row>
-    <row r="242" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>1607</v>
       </c>
@@ -20221,7 +20225,7 @@
         <v>1608</v>
       </c>
     </row>
-    <row r="243" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>1613</v>
       </c>
@@ -20277,7 +20281,7 @@
         <v>1615</v>
       </c>
     </row>
-    <row r="244" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>1619</v>
       </c>
@@ -20333,7 +20337,7 @@
         <v>1621</v>
       </c>
     </row>
-    <row r="245" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>1624</v>
       </c>
@@ -20389,7 +20393,7 @@
         <v>1626</v>
       </c>
     </row>
-    <row r="246" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>1631</v>
       </c>
@@ -20445,7 +20449,7 @@
         <v>1633</v>
       </c>
     </row>
-    <row r="247" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>1636</v>
       </c>
@@ -20501,7 +20505,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="248" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>1640</v>
       </c>
@@ -20557,7 +20561,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="249" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>1645</v>
       </c>
@@ -20610,7 +20614,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="250" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>1652</v>
       </c>
@@ -20666,7 +20670,7 @@
         <v>1656</v>
       </c>
     </row>
-    <row r="251" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>1661</v>
       </c>
@@ -20722,7 +20726,7 @@
         <v>1663</v>
       </c>
     </row>
-    <row r="252" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>1667</v>
       </c>
@@ -20778,7 +20782,7 @@
         <v>1669</v>
       </c>
     </row>
-    <row r="253" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>1673</v>
       </c>
@@ -20831,7 +20835,7 @@
         <v>1677</v>
       </c>
     </row>
-    <row r="254" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>1682</v>
       </c>
@@ -20884,7 +20888,7 @@
         <v>1685</v>
       </c>
     </row>
-    <row r="255" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>1690</v>
       </c>
@@ -20943,7 +20947,7 @@
         <v>1694</v>
       </c>
     </row>
-    <row r="256" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>1699</v>
       </c>
@@ -21002,7 +21006,7 @@
         <v>1703</v>
       </c>
     </row>
-    <row r="257" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>1708</v>
       </c>
@@ -21058,7 +21062,7 @@
         <v>1710</v>
       </c>
     </row>
-    <row r="258" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>1713</v>
       </c>
@@ -21117,7 +21121,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="259" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>1721</v>
       </c>
@@ -21173,7 +21177,7 @@
         <v>1724</v>
       </c>
     </row>
-    <row r="260" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>1729</v>
       </c>
@@ -21229,7 +21233,7 @@
         <v>1731</v>
       </c>
     </row>
-    <row r="261" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>1734</v>
       </c>
@@ -21285,7 +21289,7 @@
         <v>1737</v>
       </c>
     </row>
-    <row r="262" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>1740</v>
       </c>
@@ -21341,7 +21345,7 @@
         <v>1742</v>
       </c>
     </row>
-    <row r="263" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>1746</v>
       </c>
@@ -21397,7 +21401,7 @@
         <v>2143</v>
       </c>
     </row>
-    <row r="264" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>1751</v>
       </c>
@@ -21450,7 +21454,7 @@
         <v>1754</v>
       </c>
     </row>
-    <row r="265" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>1759</v>
       </c>
@@ -21503,7 +21507,7 @@
         <v>1762</v>
       </c>
     </row>
-    <row r="266" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>1766</v>
       </c>
@@ -21559,7 +21563,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="267" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>1775</v>
       </c>
@@ -21615,7 +21619,7 @@
         <v>1778</v>
       </c>
     </row>
-    <row r="268" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>1781</v>
       </c>
@@ -21671,7 +21675,7 @@
         <v>1783</v>
       </c>
     </row>
-    <row r="269" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>1786</v>
       </c>
@@ -21727,7 +21731,7 @@
         <v>1789</v>
       </c>
     </row>
-    <row r="270" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>1792</v>
       </c>
@@ -21783,7 +21787,7 @@
         <v>1795</v>
       </c>
     </row>
-    <row r="271" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>1798</v>
       </c>
@@ -21839,7 +21843,7 @@
         <v>1801</v>
       </c>
     </row>
-    <row r="272" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>1804</v>
       </c>
@@ -21895,7 +21899,7 @@
         <v>1807</v>
       </c>
     </row>
-    <row r="273" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>1810</v>
       </c>
@@ -21957,7 +21961,7 @@
         <v>1815</v>
       </c>
     </row>
-    <row r="274" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>1820</v>
       </c>
@@ -22013,7 +22017,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="275" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>1826</v>
       </c>
@@ -22069,7 +22073,7 @@
         <v>1829</v>
       </c>
     </row>
-    <row r="276" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>1832</v>
       </c>
@@ -22125,7 +22129,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="277" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>1838</v>
       </c>
@@ -22181,7 +22185,7 @@
         <v>1841</v>
       </c>
     </row>
-    <row r="278" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>1844</v>
       </c>
@@ -22237,7 +22241,7 @@
         <v>1847</v>
       </c>
     </row>
-    <row r="279" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>1850</v>
       </c>
@@ -22293,7 +22297,7 @@
         <v>2145</v>
       </c>
     </row>
-    <row r="280" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>1855</v>
       </c>
@@ -22349,7 +22353,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="281" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>1861</v>
       </c>
@@ -22405,7 +22409,7 @@
         <v>1864</v>
       </c>
     </row>
-    <row r="282" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>1867</v>
       </c>
@@ -22461,7 +22465,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="283" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>1873</v>
       </c>
@@ -22517,7 +22521,7 @@
         <v>1876</v>
       </c>
     </row>
-    <row r="284" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>1879</v>
       </c>
@@ -22573,7 +22577,7 @@
         <v>1882</v>
       </c>
     </row>
-    <row r="285" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>1885</v>
       </c>
@@ -22629,7 +22633,7 @@
         <v>1888</v>
       </c>
     </row>
-    <row r="286" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>1891</v>
       </c>
@@ -22685,7 +22689,7 @@
         <v>2146</v>
       </c>
     </row>
-    <row r="287" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>1898</v>
       </c>
@@ -22741,7 +22745,7 @@
         <v>1901</v>
       </c>
     </row>
-    <row r="288" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>1904</v>
       </c>
@@ -22797,7 +22801,7 @@
         <v>1907</v>
       </c>
     </row>
-    <row r="289" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>1910</v>
       </c>
@@ -22853,7 +22857,7 @@
         <v>1913</v>
       </c>
     </row>
-    <row r="290" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>1916</v>
       </c>
@@ -22909,7 +22913,7 @@
         <v>2147</v>
       </c>
     </row>
-    <row r="291" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>1921</v>
       </c>
@@ -22965,7 +22969,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="292" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>1928</v>
       </c>
@@ -23021,7 +23025,7 @@
         <v>1931</v>
       </c>
     </row>
-    <row r="293" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>1934</v>
       </c>
@@ -23083,7 +23087,7 @@
         <v>1937</v>
       </c>
     </row>
-    <row r="294" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>1942</v>
       </c>
@@ -23139,7 +23143,7 @@
         <v>1945</v>
       </c>
     </row>
-    <row r="295" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>1948</v>
       </c>
@@ -23195,7 +23199,7 @@
         <v>1951</v>
       </c>
     </row>
-    <row r="296" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>1954</v>
       </c>
@@ -23251,7 +23255,7 @@
         <v>1957</v>
       </c>
     </row>
-    <row r="297" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>1960</v>
       </c>
@@ -23307,7 +23311,7 @@
         <v>1963</v>
       </c>
     </row>
-    <row r="298" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>1966</v>
       </c>
@@ -23363,7 +23367,7 @@
         <v>1969</v>
       </c>
     </row>
-    <row r="299" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>1972</v>
       </c>
@@ -23419,7 +23423,7 @@
         <v>1975</v>
       </c>
     </row>
-    <row r="300" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>1978</v>
       </c>
@@ -23475,7 +23479,7 @@
         <v>1981</v>
       </c>
     </row>
-    <row r="301" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>1984</v>
       </c>
@@ -23531,7 +23535,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="302" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>1989</v>
       </c>
@@ -23593,7 +23597,7 @@
         <v>1993</v>
       </c>
     </row>
-    <row r="303" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>1998</v>
       </c>
@@ -23649,7 +23653,7 @@
         <v>2002</v>
       </c>
     </row>
-    <row r="304" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>2007</v>
       </c>
@@ -23705,7 +23709,7 @@
         <v>2010</v>
       </c>
     </row>
-    <row r="305" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>2015</v>
       </c>
@@ -23761,7 +23765,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="306" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>2023</v>
       </c>
@@ -23817,7 +23821,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="307" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>2082</v>
       </c>
@@ -23846,7 +23850,7 @@
         <v>2150</v>
       </c>
     </row>
-    <row r="308" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>2030</v>
       </c>
@@ -23902,7 +23906,7 @@
         <v>2151</v>
       </c>
     </row>
-    <row r="309" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>2083</v>
       </c>
@@ -23931,7 +23935,7 @@
         <v>2152</v>
       </c>
     </row>
-    <row r="310" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>2037</v>
       </c>
@@ -23987,7 +23991,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="311" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>2084</v>
       </c>
@@ -24016,7 +24020,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="312" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>2044</v>
       </c>
@@ -24072,7 +24076,7 @@
         <v>2155</v>
       </c>
     </row>
-    <row r="313" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>2085</v>
       </c>
@@ -24101,7 +24105,7 @@
         <v>2156</v>
       </c>
     </row>
-    <row r="314" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>2051</v>
       </c>
@@ -24157,7 +24161,7 @@
         <v>2157</v>
       </c>
     </row>
-    <row r="315" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>2086</v>
       </c>
@@ -24186,7 +24190,7 @@
         <v>2158</v>
       </c>
     </row>
-    <row r="316" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>2058</v>
       </c>
@@ -24242,7 +24246,7 @@
         <v>2061</v>
       </c>
     </row>
-    <row r="317" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>2087</v>
       </c>
@@ -24271,7 +24275,7 @@
         <v>2159</v>
       </c>
     </row>
-    <row r="318" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>2065</v>
       </c>
@@ -24319,7 +24323,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S318" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:S318" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="T"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S318">
     <sortCondition ref="A1:A318"/>
   </sortState>

</xml_diff>

<commit_message>
Unfinished Updating Setup Script
</commit_message>
<xml_diff>
--- a/WVS_Dataset/WVS7_Variable_Index.xlsx
+++ b/WVS_Dataset/WVS7_Variable_Index.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\file\Usersj$\jwa349\Home\My Documents\GitHub\PSYC382_WVS7_Shiny\WVS_Dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Blob\Documents\GitHub\WorldView\WVS_Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D1D4FA-91A5-4843-BBEF-48F099E655B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F30393-2580-41CE-B508-4DC80E65CE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="260" yWindow="13000" windowWidth="21760" windowHeight="18860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -6875,9 +6875,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:T318"/>
-  <sheetFormatPr defaultColWidth="28.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="28.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="8" max="8" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" customWidth="1"/>
+    <col min="11" max="11" width="17.109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6939,7 +6945,7 @@
         <v>2088</v>
       </c>
     </row>
-    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -6986,7 +6992,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -7036,7 +7042,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -7092,7 +7098,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>49</v>
       </c>
@@ -7148,7 +7154,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -7204,7 +7210,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>63</v>
       </c>
@@ -7260,7 +7266,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>70</v>
       </c>
@@ -7316,7 +7322,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -7372,7 +7378,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>84</v>
       </c>
@@ -7428,7 +7434,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>93</v>
       </c>
@@ -7484,7 +7490,7 @@
         <v>2089</v>
       </c>
     </row>
-    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>101</v>
       </c>
@@ -7540,7 +7546,7 @@
         <v>2090</v>
       </c>
     </row>
-    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2070</v>
       </c>
@@ -7569,7 +7575,7 @@
         <v>2091</v>
       </c>
     </row>
-    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>111</v>
       </c>
@@ -7625,7 +7631,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>2071</v>
       </c>
@@ -7654,7 +7660,7 @@
         <v>2092</v>
       </c>
     </row>
-    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>118</v>
       </c>
@@ -7710,7 +7716,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2072</v>
       </c>
@@ -7739,7 +7745,7 @@
         <v>2093</v>
       </c>
     </row>
-    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>125</v>
       </c>
@@ -7795,7 +7801,7 @@
         <v>2094</v>
       </c>
     </row>
-    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>2073</v>
       </c>
@@ -7824,7 +7830,7 @@
         <v>2095</v>
       </c>
     </row>
-    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>132</v>
       </c>
@@ -7880,7 +7886,7 @@
         <v>2096</v>
       </c>
     </row>
-    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>2074</v>
       </c>
@@ -7909,7 +7915,7 @@
         <v>2097</v>
       </c>
     </row>
-    <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>140</v>
       </c>
@@ -7965,7 +7971,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>2075</v>
       </c>
@@ -7994,7 +8000,7 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>147</v>
       </c>
@@ -8056,7 +8062,7 @@
         <v>2099</v>
       </c>
     </row>
-    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>160</v>
       </c>
@@ -8118,7 +8124,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>168</v>
       </c>
@@ -8180,7 +8186,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="27" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>176</v>
       </c>
@@ -8242,7 +8248,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="28" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>184</v>
       </c>
@@ -8298,7 +8304,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="29" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>189</v>
       </c>
@@ -8360,7 +8366,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="30" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>199</v>
       </c>
@@ -8422,7 +8428,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="31" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>208</v>
       </c>
@@ -8484,7 +8490,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>218</v>
       </c>
@@ -8540,7 +8546,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="33" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>227</v>
       </c>
@@ -8596,7 +8602,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>233</v>
       </c>
@@ -8652,7 +8658,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>239</v>
       </c>
@@ -8708,7 +8714,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>245</v>
       </c>
@@ -8764,7 +8770,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>251</v>
       </c>
@@ -8817,7 +8823,7 @@
         <v>2101</v>
       </c>
     </row>
-    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>259</v>
       </c>
@@ -8870,7 +8876,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>267</v>
       </c>
@@ -8926,7 +8932,7 @@
         <v>2102</v>
       </c>
     </row>
-    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>273</v>
       </c>
@@ -8985,7 +8991,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>283</v>
       </c>
@@ -9038,7 +9044,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="42" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>292</v>
       </c>
@@ -9094,7 +9100,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="43" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>301</v>
       </c>
@@ -9150,7 +9156,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="44" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>307</v>
       </c>
@@ -9206,7 +9212,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="45" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>313</v>
       </c>
@@ -9262,7 +9268,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="46" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>319</v>
       </c>
@@ -9318,7 +9324,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>325</v>
       </c>
@@ -9374,7 +9380,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>331</v>
       </c>
@@ -9430,7 +9436,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>337</v>
       </c>
@@ -9486,7 +9492,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="50" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>343</v>
       </c>
@@ -9542,7 +9548,7 @@
         <v>2103</v>
       </c>
     </row>
-    <row r="51" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>348</v>
       </c>
@@ -9595,7 +9601,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="52" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>355</v>
       </c>
@@ -9648,7 +9654,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="53" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>364</v>
       </c>
@@ -9704,7 +9710,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="54" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>373</v>
       </c>
@@ -9760,7 +9766,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="55" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>379</v>
       </c>
@@ -9816,7 +9822,7 @@
         <v>2104</v>
       </c>
     </row>
-    <row r="56" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>385</v>
       </c>
@@ -9872,7 +9878,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="57" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>391</v>
       </c>
@@ -9928,7 +9934,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>397</v>
       </c>
@@ -9984,7 +9990,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>403</v>
       </c>
@@ -10040,7 +10046,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="60" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>409</v>
       </c>
@@ -10096,7 +10102,7 @@
         <v>2105</v>
       </c>
     </row>
-    <row r="61" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>419</v>
       </c>
@@ -10152,7 +10158,7 @@
         <v>2106</v>
       </c>
     </row>
-    <row r="62" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>424</v>
       </c>
@@ -10208,7 +10214,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="63" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>430</v>
       </c>
@@ -10264,7 +10270,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="64" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>436</v>
       </c>
@@ -10320,7 +10326,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="65" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>445</v>
       </c>
@@ -10376,7 +10382,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="66" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>451</v>
       </c>
@@ -10432,7 +10438,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="67" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>458</v>
       </c>
@@ -10488,7 +10494,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="68" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>463</v>
       </c>
@@ -10544,7 +10550,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>469</v>
       </c>
@@ -10600,7 +10606,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="70" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>475</v>
       </c>
@@ -10656,7 +10662,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="71" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>482</v>
       </c>
@@ -10709,7 +10715,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="72" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>489</v>
       </c>
@@ -10765,7 +10771,7 @@
         <v>2107</v>
       </c>
     </row>
-    <row r="73" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>494</v>
       </c>
@@ -10818,7 +10824,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="74" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>500</v>
       </c>
@@ -10871,7 +10877,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="75" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>506</v>
       </c>
@@ -10927,7 +10933,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="76" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>516</v>
       </c>
@@ -10983,7 +10989,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="77" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>523</v>
       </c>
@@ -11036,7 +11042,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="78" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>530</v>
       </c>
@@ -11089,7 +11095,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="79" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>537</v>
       </c>
@@ -11142,7 +11148,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="80" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>544</v>
       </c>
@@ -11195,7 +11201,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="81" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>551</v>
       </c>
@@ -11257,7 +11263,7 @@
         <v>2108</v>
       </c>
     </row>
-    <row r="82" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>563</v>
       </c>
@@ -11319,7 +11325,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>570</v>
       </c>
@@ -11375,7 +11381,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>576</v>
       </c>
@@ -11437,7 +11443,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>582</v>
       </c>
@@ -11499,7 +11505,7 @@
         <v>2110</v>
       </c>
     </row>
-    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>588</v>
       </c>
@@ -11561,7 +11567,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>594</v>
       </c>
@@ -11620,7 +11626,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>604</v>
       </c>
@@ -11679,7 +11685,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>615</v>
       </c>
@@ -11696,7 +11702,7 @@
         <v>618</v>
       </c>
       <c r="G89" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H89" t="s">
         <v>619</v>
@@ -11735,7 +11741,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>623</v>
       </c>
@@ -11752,7 +11758,7 @@
         <v>625</v>
       </c>
       <c r="G90" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H90" t="s">
         <v>619</v>
@@ -11791,7 +11797,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>629</v>
       </c>
@@ -11808,7 +11814,7 @@
         <v>631</v>
       </c>
       <c r="G91" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H91" t="s">
         <v>619</v>
@@ -11847,7 +11853,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>635</v>
       </c>
@@ -11864,7 +11870,7 @@
         <v>637</v>
       </c>
       <c r="G92" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H92" t="s">
         <v>619</v>
@@ -11903,7 +11909,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="93" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>641</v>
       </c>
@@ -11959,7 +11965,7 @@
         <v>2111</v>
       </c>
     </row>
-    <row r="94" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>649</v>
       </c>
@@ -12015,7 +12021,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="95" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>654</v>
       </c>
@@ -12071,7 +12077,7 @@
         <v>2113</v>
       </c>
     </row>
-    <row r="96" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>659</v>
       </c>
@@ -12124,7 +12130,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="97" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>667</v>
       </c>
@@ -12177,7 +12183,7 @@
         <v>2114</v>
       </c>
     </row>
-    <row r="98" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>2076</v>
       </c>
@@ -12203,7 +12209,7 @@
         <v>2115</v>
       </c>
     </row>
-    <row r="99" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>674</v>
       </c>
@@ -12256,7 +12262,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="100" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>682</v>
       </c>
@@ -12309,7 +12315,7 @@
         <v>2116</v>
       </c>
     </row>
-    <row r="101" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>690</v>
       </c>
@@ -12362,7 +12368,7 @@
         <v>2117</v>
       </c>
     </row>
-    <row r="102" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>698</v>
       </c>
@@ -12421,7 +12427,7 @@
         <v>2118</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>708</v>
       </c>
@@ -12483,7 +12489,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>718</v>
       </c>
@@ -12545,7 +12551,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>724</v>
       </c>
@@ -12607,7 +12613,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="106" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>730</v>
       </c>
@@ -12663,7 +12669,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>738</v>
       </c>
@@ -12725,7 +12731,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>744</v>
       </c>
@@ -12787,7 +12793,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>750</v>
       </c>
@@ -12849,7 +12855,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>756</v>
       </c>
@@ -12911,7 +12917,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>762</v>
       </c>
@@ -12973,7 +12979,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>768</v>
       </c>
@@ -13035,7 +13041,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>774</v>
       </c>
@@ -13097,7 +13103,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>780</v>
       </c>
@@ -13159,7 +13165,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>786</v>
       </c>
@@ -13221,7 +13227,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>792</v>
       </c>
@@ -13283,7 +13289,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="117" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>798</v>
       </c>
@@ -13339,7 +13345,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>803</v>
       </c>
@@ -13401,7 +13407,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>809</v>
       </c>
@@ -13463,7 +13469,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>815</v>
       </c>
@@ -13525,7 +13531,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>821</v>
       </c>
@@ -13587,7 +13593,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>827</v>
       </c>
@@ -13649,7 +13655,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>834</v>
       </c>
@@ -13711,7 +13717,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="124" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>840</v>
       </c>
@@ -13767,7 +13773,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="125" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>849</v>
       </c>
@@ -13823,7 +13829,7 @@
         <v>2119</v>
       </c>
     </row>
-    <row r="126" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>855</v>
       </c>
@@ -13879,7 +13885,7 @@
         <v>2120</v>
       </c>
     </row>
-    <row r="127" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>862</v>
       </c>
@@ -13932,7 +13938,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="128" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>870</v>
       </c>
@@ -13988,7 +13994,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="129" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>875</v>
       </c>
@@ -14044,7 +14050,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="130" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>880</v>
       </c>
@@ -14097,7 +14103,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="131" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>887</v>
       </c>
@@ -14153,7 +14159,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="132" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>896</v>
       </c>
@@ -14209,7 +14215,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="133" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>903</v>
       </c>
@@ -14265,7 +14271,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="134" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>909</v>
       </c>
@@ -14321,7 +14327,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="135" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>915</v>
       </c>
@@ -14377,7 +14383,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="136" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>921</v>
       </c>
@@ -14433,7 +14439,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="137" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>927</v>
       </c>
@@ -14489,7 +14495,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="138" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>933</v>
       </c>
@@ -14545,7 +14551,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="139" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>939</v>
       </c>
@@ -14601,7 +14607,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="140" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>948</v>
       </c>
@@ -14657,7 +14663,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="141" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>953</v>
       </c>
@@ -14713,7 +14719,7 @@
         <v>2121</v>
       </c>
     </row>
-    <row r="142" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>960</v>
       </c>
@@ -14769,7 +14775,7 @@
         <v>2122</v>
       </c>
     </row>
-    <row r="143" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>966</v>
       </c>
@@ -14825,7 +14831,7 @@
         <v>2123</v>
       </c>
     </row>
-    <row r="144" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>973</v>
       </c>
@@ -14881,7 +14887,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="145" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>980</v>
       </c>
@@ -14937,7 +14943,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="146" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>986</v>
       </c>
@@ -14993,7 +14999,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="147" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>992</v>
       </c>
@@ -15049,7 +15055,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="148" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>998</v>
       </c>
@@ -15105,7 +15111,7 @@
         <v>2124</v>
       </c>
     </row>
-    <row r="149" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>1006</v>
       </c>
@@ -15161,7 +15167,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="150" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>1012</v>
       </c>
@@ -15217,7 +15223,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="151" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>1018</v>
       </c>
@@ -15273,7 +15279,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="152" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>1023</v>
       </c>
@@ -15329,7 +15335,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="153" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>1029</v>
       </c>
@@ -15385,7 +15391,7 @@
         <v>1033</v>
       </c>
     </row>
-    <row r="154" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>1038</v>
       </c>
@@ -15441,7 +15447,7 @@
         <v>2125</v>
       </c>
     </row>
-    <row r="155" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>1044</v>
       </c>
@@ -15497,7 +15503,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="156" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>1052</v>
       </c>
@@ -15553,7 +15559,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="157" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>1061</v>
       </c>
@@ -15609,7 +15615,7 @@
         <v>2126</v>
       </c>
     </row>
-    <row r="158" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>1068</v>
       </c>
@@ -15665,7 +15671,7 @@
         <v>1071</v>
       </c>
     </row>
-    <row r="159" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>1074</v>
       </c>
@@ -15721,7 +15727,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="160" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>1080</v>
       </c>
@@ -15777,7 +15783,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="161" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>1086</v>
       </c>
@@ -15833,7 +15839,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="162" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>1092</v>
       </c>
@@ -15889,7 +15895,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="163" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>1097</v>
       </c>
@@ -15945,7 +15951,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="164" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>1103</v>
       </c>
@@ -16001,7 +16007,7 @@
         <v>2127</v>
       </c>
     </row>
-    <row r="165" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>1109</v>
       </c>
@@ -16057,7 +16063,7 @@
         <v>2128</v>
       </c>
     </row>
-    <row r="166" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>1115</v>
       </c>
@@ -16113,7 +16119,7 @@
         <v>2129</v>
       </c>
     </row>
-    <row r="167" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>1121</v>
       </c>
@@ -16166,7 +16172,7 @@
         <v>2130</v>
       </c>
     </row>
-    <row r="168" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>1129</v>
       </c>
@@ -16222,7 +16228,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="169" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>1139</v>
       </c>
@@ -16278,7 +16284,7 @@
         <v>2132</v>
       </c>
     </row>
-    <row r="170" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>1145</v>
       </c>
@@ -16334,7 +16340,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="171" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>1151</v>
       </c>
@@ -16390,7 +16396,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="172" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>1157</v>
       </c>
@@ -16446,7 +16452,7 @@
         <v>2133</v>
       </c>
     </row>
-    <row r="173" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>1165</v>
       </c>
@@ -16502,7 +16508,7 @@
         <v>1167</v>
       </c>
     </row>
-    <row r="174" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>1170</v>
       </c>
@@ -16561,7 +16567,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="175" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>1178</v>
       </c>
@@ -16623,7 +16629,7 @@
         <v>1183</v>
       </c>
     </row>
-    <row r="176" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>1189</v>
       </c>
@@ -16685,7 +16691,7 @@
         <v>1192</v>
       </c>
     </row>
-    <row r="177" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>1195</v>
       </c>
@@ -16747,7 +16753,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="178" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>1202</v>
       </c>
@@ -16809,7 +16815,7 @@
         <v>1205</v>
       </c>
     </row>
-    <row r="179" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>1208</v>
       </c>
@@ -16871,7 +16877,7 @@
         <v>1211</v>
       </c>
     </row>
-    <row r="180" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>1214</v>
       </c>
@@ -16933,7 +16939,7 @@
         <v>2134</v>
       </c>
     </row>
-    <row r="181" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>1220</v>
       </c>
@@ -16995,7 +17001,7 @@
         <v>1223</v>
       </c>
     </row>
-    <row r="182" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>1226</v>
       </c>
@@ -17057,7 +17063,7 @@
         <v>1229</v>
       </c>
     </row>
-    <row r="183" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>1232</v>
       </c>
@@ -17119,7 +17125,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="184" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>1238</v>
       </c>
@@ -17175,7 +17181,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="185" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>1243</v>
       </c>
@@ -17234,7 +17240,7 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="186" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>1253</v>
       </c>
@@ -17293,7 +17299,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="187" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>1263</v>
       </c>
@@ -17352,7 +17358,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="188" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>1273</v>
       </c>
@@ -17405,7 +17411,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="189" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>1281</v>
       </c>
@@ -17464,7 +17470,7 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="190" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>1290</v>
       </c>
@@ -17526,7 +17532,7 @@
         <v>1294</v>
       </c>
     </row>
-    <row r="191" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>1299</v>
       </c>
@@ -17588,7 +17594,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="192" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>1305</v>
       </c>
@@ -17650,7 +17656,7 @@
         <v>1308</v>
       </c>
     </row>
-    <row r="193" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>1311</v>
       </c>
@@ -17712,7 +17718,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="194" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>1317</v>
       </c>
@@ -17774,7 +17780,7 @@
         <v>1320</v>
       </c>
     </row>
-    <row r="195" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>1324</v>
       </c>
@@ -17830,7 +17836,7 @@
         <v>1326</v>
       </c>
     </row>
-    <row r="196" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>1329</v>
       </c>
@@ -17844,7 +17850,7 @@
         <v>1332</v>
       </c>
       <c r="G196" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H196" t="s">
         <v>619</v>
@@ -17883,7 +17889,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="197" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>1337</v>
       </c>
@@ -17936,7 +17942,7 @@
         <v>1339</v>
       </c>
     </row>
-    <row r="198" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>1344</v>
       </c>
@@ -17950,7 +17956,7 @@
         <v>1346</v>
       </c>
       <c r="G198" t="s">
-        <v>41</v>
+        <v>153</v>
       </c>
       <c r="H198" t="s">
         <v>619</v>
@@ -17965,7 +17971,7 @@
         <v>153</v>
       </c>
       <c r="L198" t="s">
-        <v>2165</v>
+        <v>153</v>
       </c>
       <c r="M198" t="s">
         <v>1346</v>
@@ -17989,7 +17995,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="199" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>1351</v>
       </c>
@@ -18003,7 +18009,7 @@
         <v>1353</v>
       </c>
       <c r="G199" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H199" t="s">
         <v>619</v>
@@ -18042,7 +18048,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="200" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>1359</v>
       </c>
@@ -18095,7 +18101,7 @@
         <v>1362</v>
       </c>
     </row>
-    <row r="201" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>1367</v>
       </c>
@@ -18148,7 +18154,7 @@
         <v>1370</v>
       </c>
     </row>
-    <row r="202" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>1374</v>
       </c>
@@ -18198,7 +18204,7 @@
         <v>1378</v>
       </c>
     </row>
-    <row r="203" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>1381</v>
       </c>
@@ -18248,7 +18254,7 @@
         <v>1385</v>
       </c>
     </row>
-    <row r="204" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>1388</v>
       </c>
@@ -18298,7 +18304,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="205" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>1395</v>
       </c>
@@ -18351,7 +18357,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="206" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>1401</v>
       </c>
@@ -18407,7 +18413,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="207" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>1409</v>
       </c>
@@ -18460,7 +18466,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="208" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>1417</v>
       </c>
@@ -18513,7 +18519,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="209" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>1425</v>
       </c>
@@ -18569,7 +18575,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="210" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>1431</v>
       </c>
@@ -18622,7 +18628,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="211" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>1439</v>
       </c>
@@ -18675,7 +18681,7 @@
         <v>1442</v>
       </c>
     </row>
-    <row r="212" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>1447</v>
       </c>
@@ -18728,7 +18734,7 @@
         <v>1450</v>
       </c>
     </row>
-    <row r="213" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>2077</v>
       </c>
@@ -18754,7 +18760,7 @@
         <v>2135</v>
       </c>
     </row>
-    <row r="214" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>1454</v>
       </c>
@@ -18807,7 +18813,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="215" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>2078</v>
       </c>
@@ -18833,7 +18839,7 @@
         <v>2136</v>
       </c>
     </row>
-    <row r="216" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>1461</v>
       </c>
@@ -18886,7 +18892,7 @@
         <v>1464</v>
       </c>
     </row>
-    <row r="217" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>2079</v>
       </c>
@@ -18912,7 +18918,7 @@
         <v>2137</v>
       </c>
     </row>
-    <row r="218" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>1467</v>
       </c>
@@ -18965,7 +18971,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="219" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>2080</v>
       </c>
@@ -18991,7 +18997,7 @@
         <v>2138</v>
       </c>
     </row>
-    <row r="220" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>1473</v>
       </c>
@@ -19044,7 +19050,7 @@
         <v>1476</v>
       </c>
     </row>
-    <row r="221" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>1481</v>
       </c>
@@ -19100,7 +19106,7 @@
         <v>1483</v>
       </c>
     </row>
-    <row r="222" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>1486</v>
       </c>
@@ -19153,7 +19159,7 @@
         <v>1489</v>
       </c>
     </row>
-    <row r="223" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>1493</v>
       </c>
@@ -19206,7 +19212,7 @@
         <v>1496</v>
       </c>
     </row>
-    <row r="224" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>1500</v>
       </c>
@@ -19259,7 +19265,7 @@
         <v>1503</v>
       </c>
     </row>
-    <row r="225" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>1506</v>
       </c>
@@ -19312,7 +19318,7 @@
         <v>1509</v>
       </c>
     </row>
-    <row r="226" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>1511</v>
       </c>
@@ -19365,7 +19371,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="227" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>1519</v>
       </c>
@@ -19418,7 +19424,7 @@
         <v>1522</v>
       </c>
     </row>
-    <row r="228" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>1524</v>
       </c>
@@ -19471,7 +19477,7 @@
         <v>1527</v>
       </c>
     </row>
-    <row r="229" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>1532</v>
       </c>
@@ -19524,7 +19530,7 @@
         <v>1535</v>
       </c>
     </row>
-    <row r="230" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>1540</v>
       </c>
@@ -19553,7 +19559,7 @@
         <v>1</v>
       </c>
       <c r="K230" t="s">
-        <v>153</v>
+        <v>41</v>
       </c>
       <c r="L230" t="s">
         <v>2165</v>
@@ -19583,7 +19589,7 @@
         <v>1544</v>
       </c>
     </row>
-    <row r="231" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>2081</v>
       </c>
@@ -19612,7 +19618,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="232" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>1549</v>
       </c>
@@ -19668,7 +19674,7 @@
         <v>2140</v>
       </c>
     </row>
-    <row r="233" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>1552</v>
       </c>
@@ -19724,7 +19730,7 @@
         <v>1554</v>
       </c>
     </row>
-    <row r="234" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>1557</v>
       </c>
@@ -19777,7 +19783,7 @@
         <v>2141</v>
       </c>
     </row>
-    <row r="235" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>1565</v>
       </c>
@@ -19833,7 +19839,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="236" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>1570</v>
       </c>
@@ -19889,7 +19895,7 @@
         <v>1572</v>
       </c>
     </row>
-    <row r="237" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>1575</v>
       </c>
@@ -19945,7 +19951,7 @@
         <v>1577</v>
       </c>
     </row>
-    <row r="238" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>1581</v>
       </c>
@@ -20001,7 +20007,7 @@
         <v>1583</v>
       </c>
     </row>
-    <row r="239" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>1586</v>
       </c>
@@ -20057,7 +20063,7 @@
         <v>1589</v>
       </c>
     </row>
-    <row r="240" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>1594</v>
       </c>
@@ -20113,7 +20119,7 @@
         <v>1596</v>
       </c>
     </row>
-    <row r="241" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>1600</v>
       </c>
@@ -20169,7 +20175,7 @@
         <v>1602</v>
       </c>
     </row>
-    <row r="242" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>1607</v>
       </c>
@@ -20225,7 +20231,7 @@
         <v>1608</v>
       </c>
     </row>
-    <row r="243" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>1613</v>
       </c>
@@ -20281,7 +20287,7 @@
         <v>1615</v>
       </c>
     </row>
-    <row r="244" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>1619</v>
       </c>
@@ -20337,7 +20343,7 @@
         <v>1621</v>
       </c>
     </row>
-    <row r="245" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>1624</v>
       </c>
@@ -20393,7 +20399,7 @@
         <v>1626</v>
       </c>
     </row>
-    <row r="246" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>1631</v>
       </c>
@@ -20449,7 +20455,7 @@
         <v>1633</v>
       </c>
     </row>
-    <row r="247" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>1636</v>
       </c>
@@ -20505,7 +20511,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="248" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>1640</v>
       </c>
@@ -20561,7 +20567,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="249" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>1645</v>
       </c>
@@ -20614,7 +20620,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="250" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>1652</v>
       </c>
@@ -20670,7 +20676,7 @@
         <v>1656</v>
       </c>
     </row>
-    <row r="251" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>1661</v>
       </c>
@@ -20726,7 +20732,7 @@
         <v>1663</v>
       </c>
     </row>
-    <row r="252" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>1667</v>
       </c>
@@ -20782,7 +20788,7 @@
         <v>1669</v>
       </c>
     </row>
-    <row r="253" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>1673</v>
       </c>
@@ -20835,7 +20841,7 @@
         <v>1677</v>
       </c>
     </row>
-    <row r="254" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>1682</v>
       </c>
@@ -20888,7 +20894,7 @@
         <v>1685</v>
       </c>
     </row>
-    <row r="255" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>1690</v>
       </c>
@@ -20947,7 +20953,7 @@
         <v>1694</v>
       </c>
     </row>
-    <row r="256" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>1699</v>
       </c>
@@ -21006,7 +21012,7 @@
         <v>1703</v>
       </c>
     </row>
-    <row r="257" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>1708</v>
       </c>
@@ -21062,7 +21068,7 @@
         <v>1710</v>
       </c>
     </row>
-    <row r="258" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>1713</v>
       </c>
@@ -21121,7 +21127,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="259" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>1721</v>
       </c>
@@ -21177,7 +21183,7 @@
         <v>1724</v>
       </c>
     </row>
-    <row r="260" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>1729</v>
       </c>
@@ -21233,7 +21239,7 @@
         <v>1731</v>
       </c>
     </row>
-    <row r="261" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>1734</v>
       </c>
@@ -21289,7 +21295,7 @@
         <v>1737</v>
       </c>
     </row>
-    <row r="262" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>1740</v>
       </c>
@@ -21345,7 +21351,7 @@
         <v>1742</v>
       </c>
     </row>
-    <row r="263" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>1746</v>
       </c>
@@ -21401,7 +21407,7 @@
         <v>2143</v>
       </c>
     </row>
-    <row r="264" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>1751</v>
       </c>
@@ -21454,7 +21460,7 @@
         <v>1754</v>
       </c>
     </row>
-    <row r="265" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>1759</v>
       </c>
@@ -21507,7 +21513,7 @@
         <v>1762</v>
       </c>
     </row>
-    <row r="266" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>1766</v>
       </c>
@@ -21563,7 +21569,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="267" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>1775</v>
       </c>
@@ -21619,7 +21625,7 @@
         <v>1778</v>
       </c>
     </row>
-    <row r="268" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>1781</v>
       </c>
@@ -21675,7 +21681,7 @@
         <v>1783</v>
       </c>
     </row>
-    <row r="269" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>1786</v>
       </c>
@@ -21731,7 +21737,7 @@
         <v>1789</v>
       </c>
     </row>
-    <row r="270" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>1792</v>
       </c>
@@ -21787,7 +21793,7 @@
         <v>1795</v>
       </c>
     </row>
-    <row r="271" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>1798</v>
       </c>
@@ -21843,7 +21849,7 @@
         <v>1801</v>
       </c>
     </row>
-    <row r="272" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>1804</v>
       </c>
@@ -21899,7 +21905,7 @@
         <v>1807</v>
       </c>
     </row>
-    <row r="273" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>1810</v>
       </c>
@@ -21961,7 +21967,7 @@
         <v>1815</v>
       </c>
     </row>
-    <row r="274" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>1820</v>
       </c>
@@ -22017,7 +22023,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="275" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>1826</v>
       </c>
@@ -22073,7 +22079,7 @@
         <v>1829</v>
       </c>
     </row>
-    <row r="276" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>1832</v>
       </c>
@@ -22129,7 +22135,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="277" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>1838</v>
       </c>
@@ -22185,7 +22191,7 @@
         <v>1841</v>
       </c>
     </row>
-    <row r="278" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>1844</v>
       </c>
@@ -22241,7 +22247,7 @@
         <v>1847</v>
       </c>
     </row>
-    <row r="279" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>1850</v>
       </c>
@@ -22297,7 +22303,7 @@
         <v>2145</v>
       </c>
     </row>
-    <row r="280" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>1855</v>
       </c>
@@ -22353,7 +22359,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="281" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>1861</v>
       </c>
@@ -22409,7 +22415,7 @@
         <v>1864</v>
       </c>
     </row>
-    <row r="282" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>1867</v>
       </c>
@@ -22465,7 +22471,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="283" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>1873</v>
       </c>
@@ -22521,7 +22527,7 @@
         <v>1876</v>
       </c>
     </row>
-    <row r="284" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>1879</v>
       </c>
@@ -22577,7 +22583,7 @@
         <v>1882</v>
       </c>
     </row>
-    <row r="285" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>1885</v>
       </c>
@@ -22633,7 +22639,7 @@
         <v>1888</v>
       </c>
     </row>
-    <row r="286" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>1891</v>
       </c>
@@ -22689,7 +22695,7 @@
         <v>2146</v>
       </c>
     </row>
-    <row r="287" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>1898</v>
       </c>
@@ -22745,7 +22751,7 @@
         <v>1901</v>
       </c>
     </row>
-    <row r="288" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>1904</v>
       </c>
@@ -22801,7 +22807,7 @@
         <v>1907</v>
       </c>
     </row>
-    <row r="289" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>1910</v>
       </c>
@@ -22857,7 +22863,7 @@
         <v>1913</v>
       </c>
     </row>
-    <row r="290" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>1916</v>
       </c>
@@ -22913,7 +22919,7 @@
         <v>2147</v>
       </c>
     </row>
-    <row r="291" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>1921</v>
       </c>
@@ -22969,7 +22975,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="292" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>1928</v>
       </c>
@@ -23025,7 +23031,7 @@
         <v>1931</v>
       </c>
     </row>
-    <row r="293" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>1934</v>
       </c>
@@ -23087,7 +23093,7 @@
         <v>1937</v>
       </c>
     </row>
-    <row r="294" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>1942</v>
       </c>
@@ -23143,7 +23149,7 @@
         <v>1945</v>
       </c>
     </row>
-    <row r="295" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>1948</v>
       </c>
@@ -23199,7 +23205,7 @@
         <v>1951</v>
       </c>
     </row>
-    <row r="296" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>1954</v>
       </c>
@@ -23255,7 +23261,7 @@
         <v>1957</v>
       </c>
     </row>
-    <row r="297" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>1960</v>
       </c>
@@ -23311,7 +23317,7 @@
         <v>1963</v>
       </c>
     </row>
-    <row r="298" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>1966</v>
       </c>
@@ -23367,7 +23373,7 @@
         <v>1969</v>
       </c>
     </row>
-    <row r="299" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>1972</v>
       </c>
@@ -23423,7 +23429,7 @@
         <v>1975</v>
       </c>
     </row>
-    <row r="300" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>1978</v>
       </c>
@@ -23479,7 +23485,7 @@
         <v>1981</v>
       </c>
     </row>
-    <row r="301" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>1984</v>
       </c>
@@ -23535,7 +23541,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="302" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>1989</v>
       </c>
@@ -23597,7 +23603,7 @@
         <v>1993</v>
       </c>
     </row>
-    <row r="303" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>1998</v>
       </c>
@@ -23653,7 +23659,7 @@
         <v>2002</v>
       </c>
     </row>
-    <row r="304" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2007</v>
       </c>
@@ -23709,7 +23715,7 @@
         <v>2010</v>
       </c>
     </row>
-    <row r="305" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2015</v>
       </c>
@@ -23765,7 +23771,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="306" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2023</v>
       </c>
@@ -23821,7 +23827,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="307" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2082</v>
       </c>
@@ -23850,7 +23856,7 @@
         <v>2150</v>
       </c>
     </row>
-    <row r="308" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2030</v>
       </c>
@@ -23906,7 +23912,7 @@
         <v>2151</v>
       </c>
     </row>
-    <row r="309" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>2083</v>
       </c>
@@ -23935,7 +23941,7 @@
         <v>2152</v>
       </c>
     </row>
-    <row r="310" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>2037</v>
       </c>
@@ -23991,7 +23997,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="311" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>2084</v>
       </c>
@@ -24020,7 +24026,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="312" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>2044</v>
       </c>
@@ -24076,7 +24082,7 @@
         <v>2155</v>
       </c>
     </row>
-    <row r="313" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>2085</v>
       </c>
@@ -24105,7 +24111,7 @@
         <v>2156</v>
       </c>
     </row>
-    <row r="314" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>2051</v>
       </c>
@@ -24161,7 +24167,7 @@
         <v>2157</v>
       </c>
     </row>
-    <row r="315" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>2086</v>
       </c>
@@ -24190,7 +24196,7 @@
         <v>2158</v>
       </c>
     </row>
-    <row r="316" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>2058</v>
       </c>
@@ -24246,7 +24252,7 @@
         <v>2061</v>
       </c>
     </row>
-    <row r="317" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>2087</v>
       </c>
@@ -24275,7 +24281,7 @@
         <v>2159</v>
       </c>
     </row>
-    <row r="318" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>2065</v>
       </c>

</xml_diff>